<commit_message>
auto(CY): 3h refresh 2026-05-17T07:10Z
</commit_message>
<xml_diff>
--- a/daily_report_2026-05-17.xlsx
+++ b/daily_report_2026-05-17.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Removed Today" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Re-Advertisers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="New Ads Today" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="New Ads Today" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Re-Advertisers" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -559,6 +559,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Politician</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Page Name</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Page ID</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Ad ID</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>View Ad</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Ad Start</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Ad Stop</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>First Seen At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>No new ads detected today.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2142,107 +2245,4 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Politician</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Party</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>District</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>Page Name</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>Page ID</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>Ad ID</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>View Ad</t>
-        </is>
-      </c>
-      <c r="H1" s="6" t="inlineStr">
-        <is>
-          <t>Ad Start</t>
-        </is>
-      </c>
-      <c r="I1" s="6" t="inlineStr">
-        <is>
-          <t>Ad Stop</t>
-        </is>
-      </c>
-      <c r="J1" s="6" t="inlineStr">
-        <is>
-          <t>Impressions</t>
-        </is>
-      </c>
-      <c r="K1" s="6" t="inlineStr">
-        <is>
-          <t>Spend</t>
-        </is>
-      </c>
-      <c r="L1" s="6" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="M1" s="6" t="inlineStr">
-        <is>
-          <t>First Seen At</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No new ads detected today.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
auto(CY): 3h refresh 2026-05-17T13:48Z
</commit_message>
<xml_diff>
--- a/daily_report_2026-05-17.xlsx
+++ b/daily_report_2026-05-17.xlsx
@@ -456,22 +456,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -542,13 +542,386 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No ads detected as removed today.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Τσαγγάρης Ανδρέας</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Αντρέας Τσαγγάρης - ΣΗΚΟΥ ΠΑΝΩ</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>1116029114925274</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>965092452908208</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>5,000–5,999</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17 13:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ελληνας Σάββας</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Έλληνας Σάββας</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>865790916625202</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4446806865575192</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>6,000–6,999</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Λαούρης Γιάννης</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Yiannis Laouris</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>747263451806187</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>3658020847678930</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>10,000–14,999</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2387918571705884</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Αθανασιάδης Ζαχαρίας</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Ζαχαρίας Αθανασιάδης</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>146231858570802</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>1330888802244834</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>25,000–29,999</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Χαμπούλλας Ευγένιος</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>157660994287097</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3040860612787824</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>15,000–19,999</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:52</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -559,22 +932,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -645,143 +1018,34 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No new ads detected today.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="19" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Politician</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Party</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>District</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Page Name</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Page ID</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>New Ad ID</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>View Ad</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>New Ad Start</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>New Ad Stop</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Impressions</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Spend</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>First Removal Detected</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ads Removed</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Βουτηρου Σάββας</t>
+          <t>Χριστοφόρου Χριστόφορος</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Αμμόχωστος</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Σαββας Βουτήρου - Savvas Voutirou</t>
+          <t>Μωρά Θαύματα - Mora Thavmata</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>100936455330537</t>
+          <t>457092064492466</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>1299002585765427</t>
+          <t>1339492124702609</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -800,22 +1064,19 @@
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="n">
-        <v>4</v>
+          <t>2026-05-17 13:03</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Παπαδοπουλος Γεώργιος</t>
+          <t>Στυλιανού Γιάννος</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΕΔΕΚ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -825,17 +1086,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Γεώργιος Παπαδόπουλος-Georgios Papadopoulos</t>
+          <t>Στυλιανού Γιάννος</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>101463311965634</t>
+          <t>105973884902157</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>27016679577962178</t>
+          <t>1163878262531351</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -852,42 +1113,39 @@
       <c r="K3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>3</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Γεωργιάδης Δήμος</t>
+          <t>Σταύρου Σταύρος</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Κερύνεια</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Δήμος Γεωργιάδης</t>
+          <t>Zwdia.gr</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>107513542170251</t>
+          <t>108612961007638</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>1286848666896373</t>
+          <t>2188618251968315</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -897,7 +1155,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I4" s="3" t="n"/>
@@ -906,42 +1164,39 @@
       <c r="L4" s="3" t="n"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="n">
-        <v>6</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Άσπρης Άδαμος</t>
+          <t>Σταύρου Σταύρος</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Κερύνεια</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Adamos Aspris - Αδάμος Ασπρής</t>
+          <t>Zwdia.gr</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1544889622506869</t>
+          <t>108612961007638</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1287137836934355</t>
+          <t>821319647358430</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -958,42 +1213,39 @@
       <c r="K5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>2</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Άσπρης Άδαμος</t>
+          <t>Σταύρου Σταύρος</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Κερύνεια</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Adamos Aspris - Αδάμος Ασπρής</t>
+          <t>Zwdia.gr</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>1544889622506869</t>
+          <t>108612961007638</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1338561791485630</t>
+          <t>1013527524750035</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -1003,7 +1255,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="I6" s="3" t="n"/>
@@ -1012,22 +1264,19 @@
       <c r="L6" s="3" t="n"/>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="n">
-        <v>2</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Χαμπούλλας Ευγένιος</t>
+          <t>Σταύρου Σταύρος</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1037,17 +1286,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+          <t>Zwdia.gr</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>157660994287097</t>
+          <t>108612961007638</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1032725159187111</t>
+          <t>1654495512550089</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -1064,22 +1313,19 @@
       <c r="K7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>18</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Χαμπούλλας Ευγένιος</t>
+          <t>Σταύρου Σταύρος</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1089,17 +1335,17 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+          <t>Zwdia.gr</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>157660994287097</t>
+          <t>108612961007638</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>3440749736091343</t>
+          <t>1025246936697409</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -1118,42 +1364,39 @@
       <c r="L8" s="3" t="n"/>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N8" s="3" t="n">
-        <v>18</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Αποστόλου Ανδρέας</t>
+          <t>Σταύρου Σταύρος</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Λάρνακα</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ανδρέας Αποστόλου</t>
+          <t>Zwdia.gr</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>502944236549149</t>
+          <t>108612961007638</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1695784821453815</t>
+          <t>1706538184033635</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -1170,42 +1413,39 @@
       <c r="K9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>21</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Σαββίδης Χρύσανθος</t>
+          <t>Σταύρου Σταύρος</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Πάφος</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Χρύσανθος Σαββίδης</t>
+          <t>Zwdia.gr</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>556192687867978</t>
+          <t>108612961007638</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>2071083287123146</t>
+          <t>2218525365629988</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1215,7 +1455,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="I10" s="3" t="n"/>
@@ -1224,22 +1464,19 @@
       <c r="L10" s="3" t="n"/>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N10" s="3" t="n">
-        <v>27</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Σταύρου Σταύρος</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1249,17 +1486,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Zwdia.gr</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>574683626048556</t>
+          <t>108612961007638</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2460936817680213</t>
+          <t>969201902647225</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -1269,54 +1506,51 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N11" t="n">
-        <v>32</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Ευαγγελου Αργυρός</t>
+          <t>Σταύρου Σταύρος</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Λάρνακα</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Αργυρός Ευαγγέλου - Argyros Evangelou</t>
+          <t>Zwdia.gr</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>595915680800838</t>
+          <t>108612961007638</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>2039508410305874</t>
+          <t>2752559838474681</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1329,48 +1563,49 @@
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="I12" s="3" t="n"/>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
       <c r="J12" s="3" t="inlineStr"/>
       <c r="K12" s="3" t="inlineStr"/>
       <c r="L12" s="3" t="n"/>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N12" s="3" t="n">
-        <v>4</v>
+          <t>2026-05-17 13:01</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Κορύτσα Μαρία</t>
+          <t>Νεοφύτου Γιώργος</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Αμμόχωστος</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Μαρία Κορυτσά</t>
+          <t>Petra's Valley</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>636019372933735</t>
+          <t>442684272820964</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1296943101983207</t>
+          <t>1335546985122140</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -1379,11 +1614,6 @@
         </is>
       </c>
       <c r="H13" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
@@ -1392,22 +1622,19 @@
       <c r="K13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N13" t="n">
-        <v>16</v>
+          <t>2026-05-17 13:00</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Λαούρης Γιάννης</t>
+          <t>Κυριακου Δημήτρης</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>ΑΜΔΗ</t>
+          <t>ΑΛΜΑ</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1417,17 +1644,17 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Yiannis Laouris</t>
+          <t>Parasita Enterprises</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>747263451806187</t>
+          <t>580616538466482</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>978352818516825</t>
+          <t>1301553948085284</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1446,42 +1673,39 @@
       <c r="L14" s="3" t="n"/>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N14" s="3" t="n">
-        <v>13</v>
+          <t>2026-05-17 13:00</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Κυριακου Δημήτρης</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΛΜΑ</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Parasita Enterprises</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>754699914874253</t>
+          <t>580616538466482</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1271006601866511</t>
+          <t>4386862561591823</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1490,11 +1714,6 @@
         </is>
       </c>
       <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
@@ -1503,42 +1722,39 @@
       <c r="K15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N15" t="n">
-        <v>79</v>
+          <t>2026-05-17 13:00</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Κωμοδρομος Χρίστος</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΛΜΑ</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Κωμοδρόμος Χρίστος</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>754699914874253</t>
+          <t>1026160267255690</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>2150144575829086</t>
+          <t>1327096459355930</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1548,55 +1764,48 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="inlineStr"/>
       <c r="K16" s="3" t="inlineStr"/>
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N16" s="3" t="n">
-        <v>79</v>
+          <t>2026-05-17 12:57</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Παύλου Τίνα</t>
+          <t>Βουτηρου Σάββας</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Αμμόχωστος</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Τίνα Παύλου - Tina Pavlou</t>
+          <t>Σαββας Βουτήρου - Savvas Voutirou</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>802383349636152</t>
+          <t>100936455330537</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2718683645168629</t>
+          <t>1258082339646154</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1613,42 +1822,39 @@
       <c r="K17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N17" t="n">
-        <v>10</v>
+          <t>2026-05-17 12:56</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Παύλου Τίνα</t>
+          <t>Στυλιανού Μάριος</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Τίνα Παύλου - Tina Pavlou</t>
+          <t>olathrepivatis</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>802383349636152</t>
+          <t>107229495155487</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>2229818011180300</t>
+          <t>1117443331451132</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1667,22 +1873,19 @@
       <c r="L18" s="3" t="n"/>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N18" s="3" t="n">
-        <v>10</v>
+          <t>2026-05-17 12:54</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Παύλου Τίνα</t>
+          <t>Λαούρης Γιάννης</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1692,17 +1895,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Τίνα Παύλου - Tina Pavlou</t>
+          <t>Yiannis Laouris</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>802383349636152</t>
+          <t>747263451806187</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1638625114089691</t>
+          <t>1515455313465522</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -1719,42 +1922,39 @@
       <c r="K19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N19" t="n">
-        <v>10</v>
+          <t>2026-05-17 12:54</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Παύλου Τίνα</t>
+          <t>Παλιος Νίκος</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Τίνα Παύλου - Tina Pavlou</t>
+          <t>Νίκος Παλιός</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>802383349636152</t>
+          <t>97122001685</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>838326815506972</t>
+          <t>26909049372083792</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1764,55 +1964,48 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="inlineStr"/>
       <c r="K20" s="3" t="inlineStr"/>
       <c r="L20" s="3" t="n"/>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N20" s="3" t="n">
-        <v>10</v>
+          <t>2026-05-17 12:54</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Παύλου Τίνα</t>
+          <t>Παλιος Νίκος</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Τίνα Παύλου - Tina Pavlou</t>
+          <t>Νίκος Παλιός</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>802383349636152</t>
+          <t>97122001685</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1308821568004990</t>
+          <t>1340518374638199</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1822,49 +2015,46 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>10</v>
+          <t>2026-05-17 12:54</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Παύλου Τίνα</t>
+          <t>Παλιος Νίκος</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Τίνα Παύλου - Tina Pavlou</t>
+          <t>Νίκος Παλιός</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>802383349636152</t>
+          <t>97122001685</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>939589268904899</t>
+          <t>989779807335276</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1874,7 +2064,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I22" s="3" t="n"/>
@@ -1883,11 +2073,8 @@
       <c r="L22" s="3" t="n"/>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N22" s="3" t="n">
-        <v>10</v>
+          <t>2026-05-17 12:54</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -1918,7 +2105,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1173276544896604</t>
+          <t>789057964143955</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -1935,11 +2122,8 @@
       <c r="K23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>9</v>
+          <t>2026-05-17 12:54</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1970,7 +2154,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>1689103622409841</t>
+          <t>953059277706050</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1989,11 +2173,8 @@
       <c r="L24" s="3" t="n"/>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N24" s="3" t="n">
-        <v>9</v>
+          <t>2026-05-17 12:54</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -2024,7 +2205,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2115554879176833</t>
+          <t>2477463806052195</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -2041,42 +2222,39 @@
       <c r="K25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N25" t="n">
-        <v>9</v>
+          <t>2026-05-17 12:54</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Παλιος Νίκος</t>
+          <t>Κορύτσα Μαρία</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>ΑΜΔΗ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Πάφος</t>
+          <t>Αμμόχωστος</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Νίκος Παλιός</t>
+          <t>Μαρία Κορυτσά</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>97122001685</t>
+          <t>636019372933735</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>1251066740209941</t>
+          <t>2166972697493271</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -2086,7 +2264,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="I26" s="3" t="n"/>
@@ -2095,42 +2273,39 @@
       <c r="L26" s="3" t="n"/>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N26" s="3" t="n">
-        <v>9</v>
+          <t>2026-05-17 12:54</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Παλιος Νίκος</t>
+          <t>Κληρίδης Αλέξανδρος</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ΑΜΔΗ</t>
+          <t>ΔΑ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Πάφος</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Νίκος Παλιός</t>
+          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>97122001685</t>
+          <t>275808909496983</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2081720626024053</t>
+          <t>955860330696901</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -2139,11 +2314,6 @@
         </is>
       </c>
       <c r="H27" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
@@ -2152,22 +2322,19 @@
       <c r="K27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N27" t="n">
-        <v>9</v>
+          <t>2026-05-17 12:53</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Βραχιμη Έλενα</t>
+          <t>Κληρίδης Αλέξανδρος</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΠΑ</t>
+          <t>ΔΑ</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -2177,17 +2344,17 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>elena.vrachimi</t>
+          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>989853364206023</t>
+          <t>275808909496983</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>1475766074023981</t>
+          <t>1340940117880209</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -2197,7 +2364,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I28" s="3" t="n"/>
@@ -2206,11 +2373,308 @@
       <c r="L28" s="3" t="n"/>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N28" s="3" t="n">
-        <v>10</v>
+          <t>2026-05-17 12:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Κληρίδης Αλέξανδρος</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ΔΑ</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>275808909496983</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1013851890987020</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Κληρίδης Αλέξανδρος</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>ΔΑ</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>275808909496983</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>1346008437421010</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>975736668166891</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Στυλιανού Μάριος</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>ΑΛΜΑ</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Μάριος Στυλιανού</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>1007793342425297</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>1298662758901913</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="n"/>
+      <c r="J32" s="3" t="inlineStr"/>
+      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="n"/>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Αποστόλου Ανδρέας</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Λάρνακα</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Ανδρέας Αποστόλου</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>502944236549149</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1559983415752399</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Αποστόλου Ανδρέας</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Λάρνακα</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Ανδρέας Αποστόλου</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>502944236549149</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>999172072609097</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="n"/>
+      <c r="J34" s="3" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="n"/>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17 12:52</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2242,6 +2706,2676 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Politician</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Page Name</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Page ID</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>New Ad ID</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>View Ad</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>New Ad Start</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>New Ad Stop</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>First Removal Detected</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ads Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Βουτηρου Σάββας</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Αμμόχωστος</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Σαββας Βουτήρου - Savvas Voutirou</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>100936455330537</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>1299002585765427</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="inlineStr"/>
+      <c r="K2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Παπαδοπουλος Γεώργιος</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Γεώργιος Παπαδόπουλος-Georgios Papadopoulos</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>101463311965634</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>27016679577962178</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Γεωργιάδης Δήμος</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Κερύνεια</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Δήμος Γεωργιάδης</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>107513542170251</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>1286848666896373</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Άσπρης Άδαμος</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Κερύνεια</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Adamos Aspris - Αδάμος Ασπρής</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1544889622506869</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1287137836934355</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Άσπρης Άδαμος</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Κερύνεια</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Adamos Aspris - Αδάμος Ασπρής</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>1544889622506869</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>1338561791485630</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Χαμπούλλας Ευγένιος</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>157660994287097</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1032725159187111</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Χαμπούλλας Ευγένιος</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>157660994287097</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>3440749736091343</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Αποστόλου Ανδρέας</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Λάρνακα</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ανδρέας Αποστόλου</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>502944236549149</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1695784821453815</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Σαββίδης Χρύσανθος</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Χρύσανθος Σαββίδης</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>556192687867978</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>2071083287123146</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>574683626048556</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2460936817680213</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Ευαγγελου Αργυρός</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Λάρνακα</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Αργυρός Ευαγγέλου - Argyros Evangelou</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>595915680800838</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>2039508410305874</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Κορύτσα Μαρία</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Αμμόχωστος</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Μαρία Κορυτσά</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>636019372933735</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1296943101983207</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Λαούρης Γιάννης</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Yiannis Laouris</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>747263451806187</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>978352818516825</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>754699914874253</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1271006601866511</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>754699914874253</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>2150144575829086</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2718683645168629</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>2229818011180300</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="inlineStr"/>
+      <c r="K18" s="3" t="inlineStr"/>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1638625114089691</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>838326815506972</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="n"/>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1308821568004990</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>939589268904899</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="inlineStr"/>
+      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="n"/>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1173276544896604</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>1689103622409841</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr"/>
+      <c r="L24" s="3" t="n"/>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2115554879176833</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>1251066740209941</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="n"/>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2081720626024053</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Βραχιμη Έλενα</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΠΑ</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>elena.vrachimi</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>989853364206023</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>1475766074023981</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="inlineStr"/>
+      <c r="K28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="n"/>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Politician</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Page Name</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Page ID</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>New Ad ID</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>View Ad</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>New Ad Start</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>New Ad Stop</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>First Removal Detected</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Total Ads Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Στυλιανού Μάριος</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>ΑΛΜΑ</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Μάριος Στυλιανού</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>1007793342425297</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>1298662758901913</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Βουτηρου Σάββας</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Αμμόχωστος</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Σαββας Βουτήρου - Savvas Voutirou</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>100936455330537</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1258082339646154</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Κωμοδρομος Χρίστος</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>ΑΛΜΑ</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Κωμοδρόμος Χρίστος</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>1026160267255690</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>1327096459355930</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="n"/>
+      <c r="J32" s="3" t="inlineStr"/>
+      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="n"/>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Στυλιανού Γιάννος</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ΕΔΕΚ</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Στυλιανού Γιάννος</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>105973884902157</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1163878262531351</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Κληρίδης Αλέξανδρος</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>ΔΑ</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>275808909496983</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>955860330696901</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="n"/>
+      <c r="J34" s="3" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="n"/>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Κληρίδης Αλέξανδρος</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ΔΑ</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>275808909496983</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>1340940117880209</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Κληρίδης Αλέξανδρος</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>ΔΑ</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>275808909496983</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>1013851890987020</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="n"/>
+      <c r="J36" s="3" t="inlineStr"/>
+      <c r="K36" s="3" t="inlineStr"/>
+      <c r="L36" s="3" t="n"/>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="N36" s="3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Κληρίδης Αλέξανδρος</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ΔΑ</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>275808909496983</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1346008437421010</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="N37" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Αποστόλου Ανδρέας</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Λάρνακα</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Ανδρέας Αποστόλου</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>502944236549149</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>1559983415752399</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="n"/>
+      <c r="J38" s="3" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="n"/>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Αποστόλου Ανδρέας</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Λάρνακα</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Ανδρέας Αποστόλου</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>502944236549149</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>999172072609097</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Κορύτσα Μαρία</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Αμμόχωστος</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Μαρία Κορυτσά</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>636019372933735</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>2166972697493271</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="n"/>
+      <c r="J40" s="3" t="inlineStr"/>
+      <c r="K40" s="3" t="inlineStr"/>
+      <c r="L40" s="3" t="n"/>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N40" s="3" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Λαούρης Γιάννης</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Yiannis Laouris</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>747263451806187</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1515455313465522</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>975736668166891</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="n"/>
+      <c r="J42" s="3" t="inlineStr"/>
+      <c r="K42" s="3" t="inlineStr"/>
+      <c r="L42" s="3" t="n"/>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N42" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>26909049372083792</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>1340518374638199</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="n"/>
+      <c r="J44" s="3" t="inlineStr"/>
+      <c r="K44" s="3" t="inlineStr"/>
+      <c r="L44" s="3" t="n"/>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N44" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>989779807335276</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>789057964143955</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="n"/>
+      <c r="J46" s="3" t="inlineStr"/>
+      <c r="K46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="n"/>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N46" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>953059277706050</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>2477463806052195</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="n"/>
+      <c r="J48" s="3" t="inlineStr"/>
+      <c r="K48" s="3" t="inlineStr"/>
+      <c r="L48" s="3" t="n"/>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N48" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>